<commit_message>
Week 6 & 7
</commit_message>
<xml_diff>
--- a/AI_Audit_Log_NguyenThanhQuan.xlsx
+++ b/AI_Audit_Log_NguyenThanhQuan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_Uni\SU_26\SWD392\ai-audit-log-123-WaanTh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B80B860-28B9-4C61-91D9-4E1B0BE95D43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B252B73F-C945-43DD-B072-9D03ECC3F5D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,15 @@
     <sheet name="Week 3" sheetId="3" r:id="rId3"/>
     <sheet name="Week 4" sheetId="4" r:id="rId4"/>
     <sheet name="Week 5" sheetId="5" r:id="rId5"/>
+    <sheet name="Week 6" sheetId="6" r:id="rId6"/>
+    <sheet name="Week 7" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="85">
   <si>
     <t>STT</t>
   </si>
@@ -253,18 +255,124 @@
     <t>Phản hồi: AI đề xuất: xác định đối tượng → liệt kê trạng thái → xác định sự kiện → vẽ transition.
 Quyết định: Tôi bổ sung bước "xác định guard condition" và "kiểm tra tính nhất quán với Sequence Diagram" vì AI bỏ sót hai bước kiểm tra quan trọng này.</t>
   </si>
+  <si>
+    <t>State-dependent Dynamic Modeling</t>
+  </si>
+  <si>
+    <t>"State Diagram là gì và được sử dụng để làm gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích State Diagram mô tả các trạng thái của đối tượng và các sự kiện làm thay đổi trạng thái.
+Kiểm chứng: Tôi đối chiếu với slide bài học.
+Quyết định: Sử dụng State Diagram để mô hình hóa trạng thái của Ticket.</t>
+  </si>
+  <si>
+    <t>Xác định đối tượng</t>
+  </si>
+  <si>
+    <t>"Đối tượng nào trong Smart Queue Management System nên có State Diagram?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất Ticket vì đối tượng này thay đổi trạng thái theo thời gian.
+Kiểm chứng: Đối chiếu với nghiệp vụ hệ thống.
+Quyết định: Chọn Ticket để xây dựng State Diagram.</t>
+  </si>
+  <si>
+    <t>Initial State</t>
+  </si>
+  <si>
+    <t>"Trạng thái ban đầu của Ticket là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất trạng thái Created sau khi khách hàng lấy số thứ tự.
+Kiểm chứng: So sánh với quy trình nghiệp vụ.
+Quyết định: Chọn Created là trạng thái đầu tiên.</t>
+  </si>
+  <si>
+    <t>State Identification</t>
+  </si>
+  <si>
+    <t>"Ticket có thể trải qua những trạng thái nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất Created, Waiting, Called, Serving, Completed và Cancelled.
+Kiểm chứng: Đối chiếu với Use Case của nhóm.
+Quyết định: Áp dụng các trạng thái này vào sơ đồ.</t>
+  </si>
+  <si>
+    <t>Component Diagram</t>
+  </si>
+  <si>
+    <t>"Component Diagram là gì và được sử dụng trong giai đoạn nào của UML?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích Component Diagram mô tả kiến trúc vật lý của hệ thống, thể hiện các module phần mềm và mối quan hệ giữa chúng.
+Kiểm chứng: Tôi đối chiếu với slide bài học về Component Diagram.
+Quyết định: Sử dụng Component Diagram để mô tả kiến trúc của dự án nhóm.</t>
+  </si>
+  <si>
+    <t>Xác định Component</t>
+  </si>
+  <si>
+    <t>"Đối với Smart Queue Management System Using AI, hệ thống nên có những component nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các component như Mobile App, Web Dashboard, Queue Management Service, AI Prediction Service, Notification Service và Database.
+Kiểm chứng: Tôi đối chiếu với kiến trúc hệ thống mà nhóm đã xây dựng.
+Quyết định: Chọn các component phù hợp để đưa vào sơ đồ.</t>
+  </si>
+  <si>
+    <t>Front-end Component</t>
+  </si>
+  <si>
+    <t>"Frontend của hệ thống nên được biểu diễn như thế nào trong Component Diagram?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất tách thành Mobile App và Admin Dashboard vì phục vụ hai nhóm người dùng khác nhau.
+Kiểm chứng: So sánh với yêu cầu của dự án.
+Quyết định: Tách Front-end thành hai component riêng.</t>
+  </si>
+  <si>
+    <t>Backend Component</t>
+  </si>
+  <si>
+    <t>"Backend nên chia thành những component nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất Queue Service, User Service, AI Service và Notification Service để tăng tính mô-đun.
+Kiểm chứng: Đối chiếu với kiến trúc backend của nhóm.
+Quyết định: Thiết kế backend theo các service độc lập.</t>
+  </si>
+  <si>
+    <t>AI Component</t>
+  </si>
+  <si>
+    <t>"AI Prediction Service có vai trò gì trong Component Diagram?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích component này nhận dữ liệu hàng chờ và dự đoán thời gian chờ để gửi kết quả cho Queue Service.
+Kiểm chứng: Đối chiếu với chức năng AI của dự án.
+Quyết định: Thêm AI Prediction Service vào Component Diagram.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -385,9 +493,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -395,7 +503,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -404,80 +512,95 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1269,4 +1392,188 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38BB02CC-D572-442E-82CA-C4DC262408E7}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="38.44140625" customWidth="1"/>
+    <col min="3" max="3" width="32.109375" customWidth="1"/>
+    <col min="4" max="4" width="47" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="31">
+        <v>1</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="31">
+        <v>2</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="31">
+        <v>3</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="31">
+        <v>4</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5005F7A3-CD1F-4693-9348-502CD86EC53C}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="39.44140625" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="4" max="4" width="45.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="31">
+        <v>1</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="31">
+        <v>2</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="31">
+        <v>3</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="31">
+        <v>4</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="31">
+        <v>5</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>